<commit_message>
v1.2: control framing and cross-reference clarifications
Clarifications and cross-reference corrections from external review. No factors added, removed, reworded, or re-homed; all identifiers unchanged.

- Control framing: not a control standard. Factors may imply a missing or deficient control condition, but none is phrased as a control to implement.
- Cross-references: »n now marks two-faced pairs only, with both faces of all 15 pairs marked (32 markers on 30 factors, down from 35). See-also pointers moved to a new part of the Cross-references sheet (20, by ID) and no longer appear on the poster.
- Transparency pair corrected: AIRM-092 -> AIRM-093.
- Markdown corpus now carries the design principles for AI-assisted use.
- README: marker kinds, control framing, v1.2 citation and pinned links.
</commit_message>
<xml_diff>
--- a/AI-Risk-Map-Taxonomy.xlsx
+++ b/AI-Risk-Map-Taxonomy.xlsx
@@ -170,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -267,6 +267,10 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -646,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B91"/>
+  <dimension ref="A1:B93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -673,7 +677,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>v1.1 (September 2026). First public release v1.0, September 2026. Changes since are recorded at factor grain on the Change log sheet.</t>
+          <t>v1.2 (September 2026). First public release v1.0, September 2026. Changes since are recorded at factor grain on the Change log sheet.</t>
         </is>
       </c>
     </row>
@@ -757,7 +761,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>IMPORTANT: the two-faced splits. Many risks have two legitimate faces owned by different functions. This sheet lists each pair with the factor IDs on both faces, so an apparent duplicate can be checked before it is reported as one.</t>
+          <t>IMPORTANT: Part 1 lists the two-faced pairs (one risk, two owners; count once) with the factor IDs on both faces. Every »n / →n marker points to one of these pairs, so an apparent duplicate can be checked before it is reported as one. Part 2 lists one-way see-also pointers (different risks worth reading together; count both), which are not marked on the poster.</t>
         </is>
       </c>
     </row>
@@ -841,7 +845,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Risk arising from the organization's OWN ADOPTION of AI. Others' use of AI against you — AI-enabled fraud, deepfake impersonation, adversarial automation — is out of scope and belongs on the threat/cyber register. This is a boundary of subject, not degree: AI-enabled phishing passes the incremental-risk lens and is still excluded.</t>
+          <t>Risk arising from the organization's OWN ADOPTION of AI. Others' use of AI against you (AI-enabled fraud, deepfake impersonation, adversarial automation) is out of scope and belongs on the threat/cyber register. This is a boundary of subject, not degree: AI-enabled phishing passes the incremental-risk lens and is still excluded.</t>
         </is>
       </c>
     </row>
@@ -853,7 +857,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Within that boundary, only risks AI introduces or amplifies. Generic IT/cyber/vendor risk stays off.</t>
+          <t>Within that boundary, only risks AI introduces or amplifies. Generic IT, cyber, and vendor risk that exists identically without AI stays off.</t>
         </is>
       </c>
     </row>
@@ -865,7 +869,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>A factor earns its place if it clears ANY one: (A) AI-specific — remove AI and the risk vanishes; (B) management delta — the risk is not new but existing controls are insufficient for the AI version; (C) standards corroboration — two or more AI standards name it independently.</t>
+          <t>A factor earns its place if it clears ANY one: (A) AI-specific: remove AI and the risk vanishes; (B) management delta: the risk is not new, but the way it must be managed is; (C) corroboration: two or more independent AI standards name it.</t>
         </is>
       </c>
     </row>
@@ -877,777 +881,801 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>The management delta must be specific and nameable, not merely 'there is more of it.'</t>
+          <t>The management delta must be specific and nameable, not merely 'there is more of it'. 'Agent-framework sprawl outpacing credential governance' qualifies; 'cyber risk went up' does not.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Admission vs. priority</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Passing a gate is admission, not priority. When there were more good candidates than the page could hold, the tiebreak was how likely a competent team is to overlook the factor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Owner-based axis</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Domains are organized by who owns the risk, not by AI lifecycle. DASF and OWASP feed content; they do not set structure.</t>
-        </is>
-      </c>
+      <c r="B24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Two-faced risk rule</t>
+          <t>Owner-based axis</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Many AI risks have an attack face and a condition face. The attack face routes to Security or Autonomy; the condition face to the function that owns it. Cross-referenced, never duplicated. See the Cross-references sheet.</t>
+          <t>Domains are organized by who owns the risk, not by AI lifecycle. DASF and OWASP feed content; they do not set structure.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Domain routing rule</t>
+          <t>Two-faced risk rule</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>A technology pattern does not earn its own domain; its risks route to the risk type they belong to. A new domain is justified only when a risk type has no home on the axis.</t>
+          <t>Many AI risks have an attack face and a condition face, owned by different functions. The attack face routes to Security or Autonomy; the condition face to the function that owns it. The two are cross-referenced, never duplicated. See the Cross-references sheet.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
+          <t>Domain routing rule</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>A technology pattern does not earn its own domain; its risks route to the risk type they belong to. A new domain is justified only when a risk type has no home on the axis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t>Granularity calibration</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Aim for 3–4 factors per category at a consistent altitude; never pad a lean category to hit a quota. v1.0 outcome: mean 3.5 per category, range 2–6, with 48 of 54 categories at 3 or 4.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>FORM</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>What a risk factor is</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>An outcome or condition, never a control ('MFA') and never a threat actor ('an attacker').</t>
-        </is>
-      </c>
+      <c r="B29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Why 'risk factor'</t>
+          <t>What a risk factor is</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Tier 3 entries mix conditions, failure modes, threat events, and loss events. They are not well-formed loss-event statements in the FAIR sense. Scope one before using it in analysis.</t>
+          <t>A condition, failure mode, or event that contributes to risk. It may imply a missing or deficient control condition, but it is never phrased as a control to implement ('implement MFA') and never as a threat actor ('an attacker'). A proposal that arrives as a control is inverted into the condition it prevents, then checked against neighboring factors before it is added or declined.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Poster label vs description</t>
+          <t>Not a control standard</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>The workbook holds the full description; the poster holds a short label in its own column, authored not truncated. Shorten by cutting the generic stem, NOT the AI clause.</t>
+          <t>Many factors imply a missing or deficient control condition. That is deliberate: a control gap is a condition that contributes to risk. But no factor is phrased as a control to implement, and the map does not say which control closes a gap. One factor may call for several controls, and one control may address several factors. It never names threat actors.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>ARTIFACTS</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr"/>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Why 'risk factor'</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Tier 3 entries mix conditions, failure modes, threat events, and loss events. They are not well-formed loss-event statements in the FAIR sense. Scope one before using it in analysis.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Poster purpose</t>
+          <t>Poster label vs description</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>A one-page reference that widens perspective before formal assessment. Anything that helps a reader skip content works against it.</t>
+          <t>The workbook holds the full description; the poster holds a short label in its own column, authored not truncated. Shorten by cutting the generic stem, NOT the AI clause.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>Workbook purpose</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Supporting role to the poster: track provenance and enable analysis before changing the map. STOPPING RULE: not a standalone tool for scoping scenarios, running assessments, or scoring risk.</t>
-        </is>
-      </c>
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>ARTIFACTS</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>One-way generation</t>
+          <t>Poster purpose</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>The poster renders FROM this workbook. Never hand-edit the poster.</t>
+          <t>A one-page reference that widens perspective before formal assessment. Anything that helps a reader skip content works against it.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Cross-reference marker</t>
+          <t>Workbook purpose</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>On the poster, a factor with another face carries »n in the destination domain's color. Color is a wayfinding hint; the number identifies.</t>
+          <t>Supporting role to the poster: track provenance and enable analysis before changing the map. STOPPING RULE: not a standalone tool for scoping scenarios, running assessments, or scoring risk.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>PROCESS</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr"/>
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>One-way generation</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>The poster renders FROM this workbook. Never hand-edit the poster.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Four validation passes</t>
+          <t>Cross-reference markers</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>When structure changes, run in order: framework crosswalk, MECE audit, granularity calibration, lifecycle sweep. Each catches errors the others miss.</t>
+          <t>»n on the poster (→n in the X-ref column) means the other face of this risk is owned by domain n: a TWO-FACED PAIR, one underlying risk seen from two owners' chairs; count it once. The marker is used for nothing else. Both faces of every pair are marked, on at least one factor per face; the Cross-references sheet lists every factor ID on each face. SEE-ALSO POINTERS link different risks worth reading together (a more general factor, or the mirror image of the same behavior: done to you vs. done by you); count both. They are listed on the Cross-references sheet and carry no poster marker. On the poster the marker takes the destination domain's color; color is a wayfinding hint, the number identifies.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>Verify against the source</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>When a gap is claimed, check the actual source before accepting it.</t>
-        </is>
-      </c>
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Search before asserting</t>
+          <t>Four validation passes</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>AI regulation moves faster than any reference. Verify current status before citing a law, deadline, or framework version.</t>
+          <t>When structure changes, run in order: framework crosswalk, MECE audit, granularity calibration, lifecycle sweep. Each catches errors the others miss.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Provenance</t>
+          <t>Verify against the source</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Each factor tagged to its source framework(s). 'Original' = authored for this map; no reviewed framework names it. See the source-notation legend on this sheet.</t>
+          <t>When a gap is claimed, check the actual source before accepting it.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>HOW TO READ THE SOURCE(S) COLUMN</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr"/>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Search before asserting</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>AI regulation moves faster than any reference. Verify current status before citing a law, deadline, or framework version.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>NAME 0.0</t>
+          <t>Provenance</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Traces to a specific numbered element in that source (e.g. DASF 5.1, EU Art 14, OWASP LLM01).</t>
+          <t>Each factor tagged to its source framework(s). 'Original' = authored for this map; no reviewed framework names it. See the source-notation legend on this sheet.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>NAME (no number)</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>The concept appears in that source at section or theme level, not as one numbered element.</t>
-        </is>
-      </c>
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>HOW TO READ THE SOURCE(S) COLUMN</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>NAME 0.0</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Authored for this map. No reviewed framework names it.</t>
+          <t>Traces to a specific numbered element in that source (e.g. DASF 5.1, EU Art 14, OWASP LLM01).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>NAME; Original</t>
+          <t>NAME (no number)</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>The concept traces to that source; the framing and wording are ours. Named sources first, 'Original' always last.</t>
+          <t>The concept appears in that source at section or theme level, not as one numbered element.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Authored for this map. No reviewed framework names it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>NAME; Original</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>The concept traces to that source; the framing and wording are ours. Named sources first, 'Original' always last.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>v1.1 — released. Domains and categories are stable; factors change only through the Change log.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr"/>
-      <c r="B48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>v1.2 — released. Domains and categories are stable; factors change only through the Change log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr"/>
+      <c r="B50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>License and attribution</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>License</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>AI Risk Map (c) 2026 Evan Wheeler. Licensed under Creative Commons Attribution-ShareAlike 4.0 International (CC BY-SA 4.0).</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>License terms</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>https://creativecommons.org/licenses/by-sa/4.0/</t>
-        </is>
-      </c>
+      <c r="B51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>You may</t>
+          <t>License</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Share and adapt this work, including commercially.</t>
+          <t>AI Risk Map (c) 2026 Evan Wheeler. Licensed under Creative Commons Attribution-ShareAlike 4.0 International (CC BY-SA 4.0).</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>You must</t>
+          <t>License terms</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>(1) Give appropriate credit: "AI Risk Map (c) 2026 Evan Wheeler, CC BY-SA 4.0"; (2) indicate if changes were made; (3) license any adaptation under CC BY-SA 4.0.</t>
+          <t>https://creativecommons.org/licenses/by-sa/4.0/</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
+          <t>You may</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Share and adapt this work, including commercially.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>You must</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>(1) Give appropriate credit: "AI Risk Map (c) 2026 Evan Wheeler, CC BY-SA 4.0"; (2) indicate if changes were made; (3) license any adaptation under CC BY-SA 4.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
           <t>Source attribution</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Databricks AI Security Framework (DASF) v3.0 and Databricks AI Governance Framework v1.0 are (c) Databricks, licensed CC BY-SA 4.0; this work adapts material from both. The MIT AI Risk Repository is (c) MIT FutureTech, licensed CC BY 4.0; its sub-domain numbering is used in citations.</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr"/>
-      <c r="B55" s="2" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr"/>
+      <c r="B57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>Poster footnotes (rendered verbatim on the poster)</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>1. Form</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>each entry is a risk FACTOR: a condition, failure mode, or event that contributes to risk. Scope it before analysis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>2. Quantification</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>some factors scope cleanly into CRQ/FAIR scenarios; others are board-narrative.</t>
-        </is>
-      </c>
+      <c r="B58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>3. Likelihood</t>
+          <t>1. Form</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>position and size do not imply likelihood or severity; rare high-impact factors sit beside common ones.</t>
+          <t>each entry is a risk FACTOR: a condition, failure mode, or event that contributes to risk. Scope it before analysis.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>4. Use</t>
+          <t>2. Quantification</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>this map seeds threat modeling and risk assessment; it complements, it does not replace, system-specific models.</t>
+          <t>some factors scope cleanly into CRQ/FAIR scenarios; others are board-narrative.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>5. Scope</t>
+          <t>3. Likelihood</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>risks from your organization's adoption of AI; others' use of AI against you belongs on your threat register. Not exhaustive; customize to your context.</t>
+          <t>position and size do not imply likelihood or severity; rare high-impact factors sit beside common ones.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
+          <t>4. Use</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>this map seeds threat modeling and risk assessment; it complements, it does not replace, system-specific models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>5. Scope</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>risks from your organization's adoption of AI; others' use of AI against you belongs on your threat register. Not exhaustive; customize to your context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
           <t>»n</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>»n = a related factor owned by domain n, the same risk from that function's angle. Color matches the domain; full descriptions in the workbook.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr"/>
-      <c r="B63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>»n = the other face of this risk, owned by domain n; count the pair once. Color matches the domain; factor IDs for both faces are on the workbook's Cross-references sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr"/>
+      <c r="B65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>Source key</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>NIST GenAI #n</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>NIST AI 600-1 GenAI Profile — 12 risk categories</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>NIST Govern/Map/Measure/Manage</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>NIST AI RMF 1.0 — core functions</t>
-        </is>
-      </c>
+      <c r="B66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>EU Art n</t>
+          <t>NIST GenAI #n</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>EU AI Act (Reg. 2024/1689, as amended 2026) — articles; '(amended 2026)' = changed by the Digital Omnibus</t>
+          <t>NIST AI 600-1 GenAI Profile — 12 risk categories</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>GDPR</t>
+          <t>NIST Govern/Map/Measure/Manage</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>GDPR — document level</t>
+          <t>NIST AI RMF 1.0 — core functions</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>ISO A.n</t>
+          <t>EU Art n</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>ISO/IEC 42001 — Annex A control objectives</t>
+          <t>EU AI Act (Reg. 2024/1689, as amended 2026) — articles; '(amended 2026)' = changed by the Digital Omnibus</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>OWASP LLMnn</t>
+          <t>GDPR</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>OWASP Top 10 for LLM Applications 2025</t>
+          <t>GDPR — document level</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>OWASP ASI Tn</t>
+          <t>ISO A.n</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>OWASP Agentic AI — Threats &amp; Mitigations — threat IDs T1–T15 from the OWASP Agentic Security Initiative guide; the separate Top 10 for Agentic Applications numbers ASI01–ASI10</t>
+          <t>ISO/IEC 42001 — Annex A control objectives</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>OWASP AISVS n.n.n / AC.n</t>
+          <t>OWASP LLMnn</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>OWASP AISVS 1.0 — requirements; AC = Appendix C</t>
+          <t>OWASP Top 10 for LLM Applications 2025</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>OWASP</t>
+          <t>OWASP ASI Tn</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>OWASP (other)</t>
+          <t>OWASP Agentic AI — Threats &amp; Mitigations — threat IDs T1–T15 from the OWASP Agentic Security Initiative guide; the separate Top 10 for Agentic Applications numbers ASI01–ASI10</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>ATLAS AML.Tnnnn</t>
+          <t>OWASP AISVS n.n.n / AC.n</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>MITRE ATLAS — technique IDs</t>
+          <t>OWASP AISVS 1.0 — requirements; AC = Appendix C</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>DASF n.n</t>
+          <t>OWASP</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Databricks AI Security Framework v3.0 — risk IDs</t>
+          <t>OWASP (other)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Databricks AIGF</t>
+          <t>ATLAS AML.Tnnnn</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Databricks AI Governance Framework — 5 pillars</t>
+          <t>MITRE ATLAS — technique IDs</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>COSO GenAI 2026</t>
+          <t>DASF n.n</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>COSO — Internal Control over GenAI (2026) — principles</t>
+          <t>Databricks AI Security Framework v3.0 — risk IDs</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>CRI XX-n.n.n</t>
+          <t>Databricks AIGF</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>CRI Financial Services AI RMF v1.0 — control-objective IDs</t>
+          <t>Databricks AI Governance Framework — 5 pillars</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>CoSAI AI SRF</t>
+          <t>COSO GenAI 2026</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>CoSAI AI Shared Responsibility Framework — five-layer accountability model</t>
+          <t>COSO — Internal Control over GenAI (2026) — principles</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Cisco/VAIL provenance-entanglement research 2026</t>
+          <t>CRI XX-n.n.n</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Cisco / VAIL 'Models Don't Have Passports' (2026) — model-lineage fingerprinting study</t>
+          <t>CRI Financial Services AI RMF v1.0 — control-objective IDs</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>CSA AICM</t>
+          <t>CoSAI AI SRF</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>CSA AI Controls Matrix v1.1 — document level</t>
+          <t>CoSAI AI Shared Responsibility Framework — five-layer accountability model</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>CSA HF post-mortem</t>
+          <t>Cisco/VAIL provenance-entanglement research 2026</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>CSA CISO post-mortem (2026 sandbox incidents) — facts only; CC BY-NC</t>
+          <t>Cisco / VAIL 'Models Don't Have Passports' (2026) — model-lineage fingerprinting study</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>2026 sandbox-escape incidents</t>
+          <t>CSA AICM</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>2026 sandbox-escape disclosures (OpenAI / Anthropic) — public reporting</t>
+          <t>CSA AI Controls Matrix v1.1 — document level</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>MIT n.n</t>
+          <t>CSA HF post-mortem</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>MIT AI Risk Repository v4 — sub-domains; CC BY 4.0</t>
+          <t>CSA CISO post-mortem (2026 sandbox incidents) — facts only; CC BY-NC</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>IAISR</t>
+          <t>2026 sandbox-escape incidents</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>International AI Safety Report — Bengio et al.</t>
+          <t>2026 sandbox-escape disclosures (OpenAI / Anthropic) — public reporting</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Weidinger I–VI</t>
+          <t>MIT n.n</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Weidinger et al. harm taxonomy — risk areas</t>
+          <t>MIT AI Risk Repository v4 — sub-domains; CC BY 4.0</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Shelby &lt;area&gt;</t>
+          <t>IAISR</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Shelby et al. sociotechnical harms</t>
+          <t>International AI Safety Report — Bengio et al.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Colorado SB/HB n</t>
+          <t>Weidinger I–VI</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Colorado AI Act / Chatbot Safety Act</t>
+          <t>Weidinger et al. harm taxonomy — risk areas</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>SR 11-7</t>
+          <t>Shelby &lt;area&gt;</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Fed SR 11-7 model risk guidance</t>
+          <t>Shelby et al. sociotechnical harms</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Cloud Risk Map analog</t>
+          <t>Colorado SB/HB n</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Cloud Risk Map (format lineage only) — structural precedent, not an AI content source</t>
+          <t>Colorado AI Act / Chatbot Safety Act</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
+          <t>SR 11-7</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Fed SR 11-7 model risk guidance</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Risk Map analog</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Cloud Risk Map (format lineage only) — structural precedent, not an AI content source</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
           <t>Original</t>
         </is>
       </c>
-      <c r="B91" s="2" t="inlineStr">
+      <c r="B93" s="2" t="inlineStr">
         <is>
           <t>Original — authored for this map — no reviewed framework names it</t>
         </is>
@@ -1917,7 +1945,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>→12</t>
+          <t>→7,12</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
@@ -1950,11 +1978,7 @@
           <t>COSO GenAI 2026; OWASP AISVS AC.8</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>→12</t>
-        </is>
-      </c>
+      <c r="G8" s="9" t="inlineStr"/>
       <c r="H8" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -2214,7 +2238,11 @@
           <t>ISO A.4; NIST Govern; CRI GV-1.6.1</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr"/>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>→4,6</t>
+        </is>
+      </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -2307,11 +2335,7 @@
           <t>COSO GenAI 2026 p.13</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>→8</t>
-        </is>
-      </c>
+      <c r="G19" s="9" t="inlineStr"/>
       <c r="H19" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -2412,7 +2436,11 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr"/>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>→11</t>
+        </is>
+      </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -2540,11 +2568,7 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>→8</t>
-        </is>
-      </c>
+      <c r="G26" s="9" t="inlineStr"/>
       <c r="H26" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -2672,11 +2696,7 @@
           <t>Databricks AIGF; CRI MP-3.2.2; Original</t>
         </is>
       </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>→11</t>
-        </is>
-      </c>
+      <c r="G30" s="9" t="inlineStr"/>
       <c r="H30" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -2909,7 +2929,11 @@
           <t>EU Art 10 (amended 2026); NIST GenAI #4</t>
         </is>
       </c>
-      <c r="G37" s="9" t="inlineStr"/>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>→5</t>
+        </is>
+      </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -3200,11 +3224,7 @@
           <t>Cloud Risk Map analog; Original</t>
         </is>
       </c>
-      <c r="G46" s="9" t="inlineStr">
-        <is>
-          <t>→8</t>
-        </is>
-      </c>
+      <c r="G46" s="9" t="inlineStr"/>
       <c r="H46" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -3794,7 +3814,11 @@
           <t>EU Art 11 (amended 2026); NIST Map</t>
         </is>
       </c>
-      <c r="G64" s="9" t="inlineStr"/>
+      <c r="G64" s="9" t="inlineStr">
+        <is>
+          <t>→1</t>
+        </is>
+      </c>
       <c r="H64" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -3992,7 +4016,11 @@
           <t>DASF 9.2 / 9.5; NIST GenAI #4</t>
         </is>
       </c>
-      <c r="G70" s="9" t="inlineStr"/>
+      <c r="G70" s="9" t="inlineStr">
+        <is>
+          <t>→3</t>
+        </is>
+      </c>
       <c r="H70" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -4384,11 +4412,7 @@
           <t>OWASP AISVS AC.13</t>
         </is>
       </c>
-      <c r="G82" s="9" t="inlineStr">
-        <is>
-          <t>→4</t>
-        </is>
-      </c>
+      <c r="G82" s="9" t="inlineStr"/>
       <c r="H82" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -4458,7 +4482,11 @@
           <t>DASF 1.1; Original</t>
         </is>
       </c>
-      <c r="G84" s="9" t="inlineStr"/>
+      <c r="G84" s="9" t="inlineStr">
+        <is>
+          <t>→12</t>
+        </is>
+      </c>
       <c r="H84" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -4520,11 +4548,7 @@
           <t>OWASP AISVS 5.2.2</t>
         </is>
       </c>
-      <c r="G86" s="9" t="inlineStr">
-        <is>
-          <t>→3</t>
-        </is>
-      </c>
+      <c r="G86" s="9" t="inlineStr"/>
       <c r="H86" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -4691,7 +4715,11 @@
           <t>NIST GenAI #3; Weidinger I</t>
         </is>
       </c>
-      <c r="G91" s="9" t="inlineStr"/>
+      <c r="G91" s="9" t="inlineStr">
+        <is>
+          <t>→5</t>
+        </is>
+      </c>
       <c r="H91" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -4792,7 +4820,11 @@
           <t>EU Art 50 (amended 2026); Weidinger V</t>
         </is>
       </c>
-      <c r="G94" s="9" t="inlineStr"/>
+      <c r="G94" s="9" t="inlineStr">
+        <is>
+          <t>→1</t>
+        </is>
+      </c>
       <c r="H94" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -5083,11 +5115,7 @@
           <t>COSO GenAI 2026; OWASP AISVS AC.4; CRI MP-3.5.4</t>
         </is>
       </c>
-      <c r="G103" s="9" t="inlineStr">
-        <is>
-          <t>→7</t>
-        </is>
-      </c>
+      <c r="G103" s="9" t="inlineStr"/>
       <c r="H103" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -5157,11 +5185,7 @@
           <t>DASF 8.3; Original</t>
         </is>
       </c>
-      <c r="G105" s="9" t="inlineStr">
-        <is>
-          <t>→1</t>
-        </is>
-      </c>
+      <c r="G105" s="9" t="inlineStr"/>
       <c r="H105" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -5254,11 +5278,7 @@
           <t>OpenAI/Anthropic 2026 incidents</t>
         </is>
       </c>
-      <c r="G108" s="9" t="inlineStr">
-        <is>
-          <t>→12</t>
-        </is>
-      </c>
+      <c r="G108" s="9" t="inlineStr"/>
       <c r="H108" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -5293,7 +5313,11 @@
           <t>DASF 10.1; NIST Manage; CSA HF post-mortem</t>
         </is>
       </c>
-      <c r="G109" s="9" t="inlineStr"/>
+      <c r="G109" s="9" t="inlineStr">
+        <is>
+          <t>→4</t>
+        </is>
+      </c>
       <c r="H109" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -5326,7 +5350,7 @@
       </c>
       <c r="G110" s="9" t="inlineStr">
         <is>
-          <t>→12</t>
+          <t>→1</t>
         </is>
       </c>
       <c r="H110" s="9" t="inlineStr">
@@ -5619,11 +5643,7 @@
           <t>CSA HF post-mortem</t>
         </is>
       </c>
-      <c r="G119" s="9" t="inlineStr">
-        <is>
-          <t>→9</t>
-        </is>
-      </c>
+      <c r="G119" s="9" t="inlineStr"/>
       <c r="H119" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -5658,11 +5678,7 @@
           <t>COSO GenAI 2026; OWASP AISVS 3.2.3; Original</t>
         </is>
       </c>
-      <c r="G120" s="9" t="inlineStr">
-        <is>
-          <t>→9</t>
-        </is>
-      </c>
+      <c r="G120" s="9" t="inlineStr"/>
       <c r="H120" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -5786,11 +5802,7 @@
           <t>2026 sandbox-escape incidents; Original</t>
         </is>
       </c>
-      <c r="G124" s="9" t="inlineStr">
-        <is>
-          <t>→1</t>
-        </is>
-      </c>
+      <c r="G124" s="9" t="inlineStr"/>
       <c r="H124" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -6050,7 +6062,11 @@
           <t>NIST GenAI #10; Original</t>
         </is>
       </c>
-      <c r="G132" s="9" t="inlineStr"/>
+      <c r="G132" s="9" t="inlineStr">
+        <is>
+          <t>→3</t>
+        </is>
+      </c>
       <c r="H132" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -6147,11 +6163,7 @@
           <t>Databricks AIGF; Original</t>
         </is>
       </c>
-      <c r="G135" s="9" t="inlineStr">
-        <is>
-          <t>→9</t>
-        </is>
-      </c>
+      <c r="G135" s="9" t="inlineStr"/>
       <c r="H135" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -6349,7 +6361,11 @@
           <t>IAISR; Original</t>
         </is>
       </c>
-      <c r="G141" s="9" t="inlineStr"/>
+      <c r="G141" s="9" t="inlineStr">
+        <is>
+          <t>→11</t>
+        </is>
+      </c>
       <c r="H141" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -6380,11 +6396,7 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="G142" s="9" t="inlineStr">
-        <is>
-          <t>→7</t>
-        </is>
-      </c>
+      <c r="G142" s="9" t="inlineStr"/>
       <c r="H142" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -6450,11 +6462,7 @@
           <t>CRI GV-6.1.1; Original</t>
         </is>
       </c>
-      <c r="G144" s="9" t="inlineStr">
-        <is>
-          <t>→10</t>
-        </is>
-      </c>
+      <c r="G144" s="9" t="inlineStr"/>
       <c r="H144" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -7168,11 +7176,7 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="G166" s="9" t="inlineStr">
-        <is>
-          <t>→8</t>
-        </is>
-      </c>
+      <c r="G166" s="9" t="inlineStr"/>
       <c r="H166" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -7374,11 +7378,7 @@
           <t>CSA HF post-mortem; Original</t>
         </is>
       </c>
-      <c r="G172" s="9" t="inlineStr">
-        <is>
-          <t>→8</t>
-        </is>
-      </c>
+      <c r="G172" s="9" t="inlineStr"/>
       <c r="H172" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -7413,7 +7413,11 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="G173" s="9" t="inlineStr"/>
+      <c r="G173" s="9" t="inlineStr">
+        <is>
+          <t>→7</t>
+        </is>
+      </c>
       <c r="H173" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -7685,7 +7689,11 @@
           <t>OWASP ASI T9; DASF 13.9</t>
         </is>
       </c>
-      <c r="G181" s="9" t="inlineStr"/>
+      <c r="G181" s="9" t="inlineStr">
+        <is>
+          <t>→5</t>
+        </is>
+      </c>
       <c r="H181" s="9" t="inlineStr">
         <is>
           <t>active</t>
@@ -7978,7 +7986,7 @@
       </c>
       <c r="G190" s="9" t="inlineStr">
         <is>
-          <t>→1,8</t>
+          <t>→1</t>
         </is>
       </c>
       <c r="H190" s="9" t="inlineStr">
@@ -8545,12 +8553,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8846,7 +8856,7 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>AIRM-063, AIRM-092</t>
+          <t>AIRM-063, AIRM-093</t>
         </is>
       </c>
     </row>
@@ -8985,7 +8995,591 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t>SEE-ALSO POINTERS (one-way)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>Different risks worth reading together; count both. The target is either a more general factor or the mirror image of the same behavior (done to you vs. done by you). One-way, and not marked on the poster: »n is reserved for the two-faced pairs above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>From ID</t>
+        </is>
+      </c>
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>From (domain · poster label)</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="inlineStr">
+        <is>
+          <t>To ID</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <t>To (domain · poster label)</t>
+        </is>
+      </c>
+      <c r="E20" s="32" t="inlineStr">
+        <is>
+          <t>Why read them together</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-007</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>1 · Segregation of duties collapses across AI config, operation, and review</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-175</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>12 · Excessive autonomy / agency beyond intended mandate</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Where the one collapsing configure / operate / review duties is an agent, Autonomy owns the agency-beyond-mandate view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-018</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>1 · AI output relied on in financial-reporting controls without scope change</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-138</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>8 · Inability to evidence and audit AI compliance across jurisdictions (internal evidence burden)</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Once AI output sits inside a regulated control chain, the burden of evidencing that chain lands on Legal &amp; Compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-025</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>2 · Misjudged AI sourcing fork: train, fine-tune, RAG, or API</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-129</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>8 · Misclassified as deployer when fine-tuning makes you a provider</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Fine-tuning or rebranding a model can turn a deployer into a provider under the EU AI Act; the sourcing choice sets the legal role.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-029</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>2 · Hidden total cost of ownership (data, talent, integration) eroding returns</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-165</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>11 · Poor cost forecasting, because inference cost scales with usage rather than seats or provisioned capacity</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Hidden total cost of ownership shows up in Finance as usage-scaled inference cost that was never forecast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-045</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>3 · Failure to preserve prompts, outputs, and agent traces subject to litigation hold or e-discovery</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-130</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>8 · Liability for harm caused by AI decisions or outputs</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Failure to preserve prompts, outputs, and agent traces becomes litigation exposure when a claim arrives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-081</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>5 · Model-invented dependencies resolving to adversary-registered packages</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-052</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>4 · Fluent but factually incorrect output (hallucination) accepted as reliable</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>The package-name attack depends on a hallucination the model repeats reliably; the accuracy defect is owned in Model Development.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-085</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>5 · Retrieval serving content beyond the user’s own entitlements</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-039</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>3 · Inadvertent disclosure of confidential / personal data in model output (no output guardrails)</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>Retrieval beyond the user's entitlements surfaces as confidential data in model output, the Data &amp; Privacy view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-102</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>6 · Review capacity cannot scale to AI output volume, degrading oversight to rubber-stamping</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-117</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>7 · Inadequate content-moderation / trust-&amp;-safety operations at scale</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>The same volume problem at operational scale: moderation and trust-and-safety teams cannot keep pace with AI output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-104</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>7 · Inconsistent or unsanctioned (shadow) model deployment</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-002</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>1 · Ungoverned ‘shadow AI’ adoption outside sanctioned channels</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Shadow deployment in Operations is the production end of shadow AI adoption, which Governance owns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-107</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>7 · Test or sandbox containment fails and AI reaches real systems</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-174</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>12 · Agent pursues an authorized objective through unauthorized means</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>In the 2026 incidents, containment failed because the agent pursued an authorized objective through unauthorized means.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-109</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>7 · Inadequate logging of inputs, outputs, tool calls, agent decisions, and who authorized them</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-187</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>12 · Accountability gap for harm caused by autonomous action</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>Logs of who authorized an agent's action are what close the accountability gap after autonomous harm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-119</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>7 · Silent vendor / model updates changing behavior without notice</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-141</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>9 · Model deprecation or behavior change forcing unplanned migration</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>A silent model update is the operational face of provider-driven behavior change; Third-Party owns the dependency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-123</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>7 · Controls re-verified less often than the AI system changes</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-017</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>1 · Absence of independent assurance over AI control effectiveness</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>Controls re-verified less often than the system changes is an assurance gap: no independent evidence the controls still work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-134</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>8 · Violation of open-weight / model license terms</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-189</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>9 · Model's true lineage hidden behind its publisher label, so upstream flaws can't be traced</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>Open-weight license obligations can be inherited through a lineage the publisher label does not disclose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-142</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>9 · Vendor diligence missing: are prompts retained, trained on, or shared?</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-036</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>3 · Personal data used for training without consent or purpose limitation</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>Mirror image: a vendor training on your prompts and outputs without agreement, and your organization training on people's personal data without consent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-141</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>9 · Model deprecation or behavior change forcing unplanned migration</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-120</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>7 · Inadequate versioning, rollback, and change control for models</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>A forced migration has to run through versioning, rollback, and change control in Operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-163</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>10 · AI-washing: overstating capability to customers, investors, or regulators</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-130</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>8 · Liability for harm caused by AI decisions or outputs</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>Overstated AI capability invites enforcement and liability claims.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-169</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>11 · Insurance excludes AI losses, or defines 'user' as human only</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-130</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>8 · Liability for harm caused by AI decisions or outputs</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>An insurance exclusion leaves the liability for AI-caused harm uninsured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-187</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>12 · Accountability gap for harm caused by autonomous action</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-130</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>8 · Liability for harm caused by AI decisions or outputs</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>The accountability gap after autonomous harm meets Legal's general liability factor. Pointer runs specific to general, so AIRM-130 carries no return marker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-188</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>9 · No way to verify a vendor's 'AI-powered' claim before buying it</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-163</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>10 · AI-washing: overstating capability to customers, investors, or regulators</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>The buyer's side of AI capability claims; AIRM-163 is the seller's side, when your own organization overstates.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A19:E19"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9071,7 +9665,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Excluded by form; entries are risk factors — conditions and failure modes — never a control ('MFA') or a threat actor ('an attacker').</t>
+          <t>Excluded by form. Entries are risk factors (conditions, failure modes, and events), never a control to implement ('implement MFA') or a threat actor ('an attacker'). A factor may imply a missing or deficient control condition; that is in form. A proposal that arrives as a control is inverted into the condition it prevents and checked against neighboring factors before it is added or declined.</t>
         </is>
       </c>
     </row>
@@ -9323,7 +9917,7 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>SOURCE: CSA CISO post-mortem recommendation to use identifiable source IP ranges with PTR records. DECLINED: this is a CONTROL, not a risk. Excluded by form rule 3.1 — factors are outcomes or conditions, never controls.</t>
+          <t>SOURCE: CSA CISO post-mortem recommendation to use identifiable source IP ranges with PTR records. NOT YET ADDED. The recommendation is a control; inverted, the condition it prevents is outward attribution: a third party affected by your agent cannot tell whose agent acted, so it cannot notify you, and you lose your earliest external warning that an agent has escaped containment. No existing factor covers this. AIRM-111 is inward (your own telemetry), AIRM-162 is the resulting harm, AIRM-109 is your internal authorization record, and AIRM-178 is misuse of an agent's identity. Queued for consideration in a future release.</t>
         </is>
       </c>
     </row>
@@ -9335,7 +9929,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>SOURCE: CSA CISO post-mortem recommendation to stand up two separate agentic response teams (victim and perpetrator). DECLINED: a control. The underlying risks are covered by D10 'Harm to non-users and third parties', D8 'Liability for harm caused by AI decisions or outputs', and D7 incident management.</t>
+          <t>SOURCE: CSA CISO post-mortem recommendation to stand up two separate agentic response teams (victim and perpetrator). DECLINED as a separate factor. The recommendation is a control; the conditions it addresses are covered by D10 'Harm to non-users and third parties', D8 'Liability for harm caused by AI decisions or outputs', and D7 incident management.</t>
         </is>
       </c>
     </row>
@@ -9374,7 +9968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9543,6 +10137,141 @@
       <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Accountability pair added to the Cross-references sheet. It was already a recorded two-faced split in Scope decisions; the sheet had omitted it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>v1.2</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>cross-ref sheet</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-092, AIRM-093</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Transparency pair corrected. It listed AIRM-092 (harm to minors) in error; the user-disclosure face is AIRM-093 (failure to disclose AI interaction).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>v1.2</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>x-ref (pairs completed)</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-006, 015, 021, 036, 063, 069, 083, 090, 093, 108, 109, 131, 140, 170, 178</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Markers added so both faces of every two-faced pair are marked: AIRM-131 →3, 108 →4, 140 →11, 021 →11, 090 →5, 178 →5, 170 →7, 083 →12, 069 →3, 036 →5, 015 →4,6, 063 →1, 093 →1, 109 →1, 006 →7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>v1.2</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>x-ref (see-also moved)</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-007, 018, 025, 029, 045, 081, 085, 102, 104, 107, 109, 118, 119, 123, 134, 141, 163, 169, 187, 188</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Markers removed. These pointed at a related but different risk, not the other face of a pair. 19 are now listed as see-also pointers on the Cross-references sheet; AIRM-118's →9 was dropped because no factor in that domain covers it. AIRM-109's →12 and AIRM-187's →8 became see-also rows; AIRM-187 keeps its pair marker →1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>v1.2</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>cross-ref sheet</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>AIRM-142, AIRM-036</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>New see-also pointer (mirror image): a vendor training on your data without agreement, and your organization training on personal data without consent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>v1.2</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>documentation</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Control framing clarified in the Read me, Scope decisions, and markdown: not a control standard; factors may imply a missing or deficient control condition but are never phrased as a control to implement. Marker documentation now distinguishes two-faced pairs from see-also pointers. No factor wording changed.</t>
         </is>
       </c>
     </row>
@@ -9566,7 +10295,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="34" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>Taxonomy sheet and CSV — column contract, frozen at v1.0. Adding, removing, or reordering a column is a major version.</t>
         </is>
@@ -9704,7 +10433,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>'→n' = this factor has another face owned by domain n. Human wayfinding hint; the Cross-references sheet is authoritative, by ID.</t>
+          <t>'→n' = the other face of this risk is owned by domain n (the poster's »n); count the pair once. Used only for two-faced pairs. Every face of every pair carries a marker, on at least one factor of that face; the Cross-references sheet lists every factor ID on both faces, so use it, not this column, to count. See-also pointers are listed on the sheet and carry no marker.</t>
         </is>
       </c>
     </row>
@@ -9753,7 +10482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9763,53 +10492,53 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="35" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>AI Risk Map — Version History</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="36" t="inlineStr">
+      <c r="A2" s="38" t="inlineStr">
         <is>
           <t>Release-level history. Factor-level changes are on the Change log sheet. Factor counts are Tier-3 risk factors.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="37" t="inlineStr">
+      <c r="A4" s="39" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B4" s="37" t="inlineStr">
+      <c r="B4" s="39" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C4" s="37" t="inlineStr">
+      <c r="C4" s="39" t="inlineStr">
         <is>
           <t>Factors</t>
         </is>
       </c>
-      <c r="D4" s="37" t="inlineStr">
+      <c r="D4" s="39" t="inlineStr">
         <is>
           <t>Changes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="40" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="B5" s="39" t="inlineStr">
+      <c r="B5" s="41" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="C5" s="39" t="n">
+      <c r="C5" s="41" t="n">
         <v>189</v>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -9819,22 +10548,42 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="40" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
       </c>
-      <c r="B6" s="39" t="inlineStr">
+      <c r="B6" s="41" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="C6" s="39" t="n">
+      <c r="C6" s="41" t="n">
         <v>189</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Poster redesign: new typeface (Figtree), lighter header with a reading key, categories set as colored text, and cross-reference markers drawn as pills in the target domain's color. Cross-reference corrections: two markers that pointed at their own domain were removed (AIRM-046, AIRM-152), and AIRM-187 now shows both of its targets, Governance and Legal, where v1.0 printed only the first. The D1/D12 accountability pair (AIRM-006 / AIRM-187) was added to the Cross-references sheet, where it had been recorded only in Scope decisions. No factors added, removed, reworded, or re-homed; all identifiers unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="40" t="inlineStr">
+        <is>
+          <t>v1.2</t>
+        </is>
+      </c>
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="n">
+        <v>189</v>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Clarifications and cross-reference corrections from external review. Control framing: the map is not a control standard; factors may imply a missing or deficient control condition, but none is phrased as a control to implement and the map does not say which control closes a gap. Cross-references: »n now means one thing, the other face of a two-faced pair (count once). Both faces of all 15 pairs are marked, where v1.1 marked both faces of only four and left three pairs unmarked. The one-way see-also pointers that shared the same marker were moved to a new part of the Cross-references sheet (20 pointers, listed by ID) and no longer appear on the poster. The build now fails if a marker and the pair list disagree in either direction. Net: 32 markers on 30 factors, down from 35. The Transparency pair listed AIRM-092 in error; corrected to AIRM-093. The markdown corpus now carries the design principles (scope, retention gates, factor form, two-faced rule, markers). No factors added, removed, reworded, or re-homed; all identifiers unchanged.</t>
         </is>
       </c>
     </row>

</xml_diff>